<commit_message>
Force push, extracing source changes and diagram
</commit_message>
<xml_diff>
--- a/tests/Testing.xlsx
+++ b/tests/Testing.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c7d7d98c037d19b/Level 6/Cloud/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c7d7d98c037d19b/Level 6/Cloud/ACDT CW2 Updated/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{AB4D71AA-F82A-4017-8E7A-B8E1FF7AC13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F89F414D-ECF2-492D-AAA2-A975A2D08059}"/>
+  <xr:revisionPtr revIDLastSave="112" documentId="8_{AB4D71AA-F82A-4017-8E7A-B8E1FF7AC13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB2213FE-3847-47D3-9F2D-26636208F9B4}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{0FD93C22-EA38-4C55-8FBA-9A662F17215C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0FD93C22-EA38-4C55-8FBA-9A662F17215C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -152,18 +152,6 @@
     <t>test_correlation_id_for_is_deterministic_and_12_chars</t>
   </si>
   <si>
-    <t>test_extract_source_domain_from_url</t>
-  </si>
-  <si>
-    <t>test_extract_source_domain_from_text_domain</t>
-  </si>
-  <si>
-    <t>test_extract_source_domain_returns_none_when_missing_name</t>
-  </si>
-  <si>
-    <t>test_extract_source_domain_bad_url_returns_none</t>
-  </si>
-  <si>
     <t>test_read_emails_from_csv_strips_and_keeps_order</t>
   </si>
   <si>
@@ -218,12 +206,6 @@
     <t>Verify CID consistency and length</t>
   </si>
   <si>
-    <t>Extract domain from URL</t>
-  </si>
-  <si>
-    <t>Extract domain from free text</t>
-  </si>
-  <si>
     <t>Handle missing name field</t>
   </si>
   <si>
@@ -281,9 +263,6 @@
     <t>URL with subdomain</t>
   </si>
   <si>
-    <t>Text containing domain</t>
-  </si>
-  <si>
     <t>Empty name</t>
   </si>
   <si>
@@ -347,9 +326,6 @@
     <t>Hashing</t>
   </si>
   <si>
-    <t>Domain Extraction</t>
-  </si>
-  <si>
     <t>Analyst Summary</t>
   </si>
   <si>
@@ -861,7 +837,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>tests/test_main.py::test_extract_source_domain_from_url</t>
+      <t>tests/test_main.py::test_read_emails_from_csv_strips_and_keeps_order</t>
     </r>
     <r>
       <rPr>
@@ -892,6 +868,372 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tests/test_main.py::test_screen_email_polls_until_records_found</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tests/test_main.py::test_request_does_not_retry_on_non_retry_status</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tests/test_main.py::test_request_honours_retry_after_header</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tests/test_main.py::test_build_analyst_summary_counts_and_top_sources</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tests/test_main.py::test_write_summary_csv_writes_expected_layout</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">   </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">tests/test_main.py::test_write_breach_chart_png_creates_file_when_breaches_exist </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tests/test_main.py::test_write_breach_chart_png_skips_when_no_breaches</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+  </si>
+  <si>
+    <t>Source Extraction</t>
+  </si>
+  <si>
+    <t>Extract source from URL</t>
+  </si>
+  <si>
+    <t>Extract source from free text</t>
+  </si>
+  <si>
+    <t>Text containing source</t>
+  </si>
+  <si>
+    <t>test_extract_source_from_url</t>
+  </si>
+  <si>
+    <t>test_extract_source_from_text</t>
+  </si>
+  <si>
+    <t>test_extract_source_returns_none_when_missing_name</t>
+  </si>
+  <si>
+    <t>test_extract_source_bad_url_returns_none</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tests/test_main.py::test_extract_domain_from_url</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PASSED</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">       </t>
     </r>
   </si>
@@ -905,7 +1247,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>tests/test_main.py::test_extract_source_domain_from_text_domain</t>
+      <t>tests/test_main.py::test_extract_source_from_text</t>
     </r>
     <r>
       <rPr>
@@ -949,7 +1291,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>tests/test_main.py::test_extract_source_domain_returns_none_when_missing_name</t>
+      <t>tests/test_main.py::test_extract_source_returns_none_when_missing_name</t>
     </r>
     <r>
       <rPr>
@@ -993,7 +1335,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">tests/test_main.py::test_extract_source_domain_bad_url_returns_none </t>
+      <t xml:space="preserve">tests/test_main.py::test_extract_source_bad_url_returns_none </t>
     </r>
     <r>
       <rPr>
@@ -1015,348 +1357,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">   </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>tests/test_main.py::test_read_emails_from_csv_strips_and_keeps_order</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>tests/test_main.py::test_screen_email_polls_until_records_found</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>tests/test_main.py::test_request_does_not_retry_on_non_retry_status</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>tests/test_main.py::test_request_honours_retry_after_header</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>tests/test_main.py::test_build_analyst_summary_counts_and_top_sources</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>tests/test_main.py::test_write_summary_csv_writes_expected_layout</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">   </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">tests/test_main.py::test_write_breach_chart_png_creates_file_when_breaches_exist </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>tests/test_main.py::test_write_breach_chart_png_skips_when_no_breaches</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>PASSED</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
     </r>
   </si>
 </sst>
@@ -1486,20 +1486,20 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>27</xdr:row>
-      <xdr:rowOff>9525</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>1487853</xdr:colOff>
-      <xdr:row>50</xdr:row>
-      <xdr:rowOff>19663</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>3298167</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>162533</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="18" name="Picture 17">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A75BD18-A0C5-F003-BAEE-CDE521BA8618}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58C4BEC0-A8AD-8244-2FDB-36038662FAB9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1515,8 +1515,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="5153025"/>
-          <a:ext cx="13994178" cy="4391638"/>
+          <a:off x="0" y="5143500"/>
+          <a:ext cx="18033342" cy="4353533"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1878,13 +1878,13 @@
         <v>6</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="6" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -1902,22 +1902,22 @@
         <v>2</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="G3" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I3" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1931,22 +1931,22 @@
         <v>2</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="G4" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I4" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -1957,25 +1957,25 @@
         <v>30</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" t="s">
         <v>48</v>
       </c>
-      <c r="E5" t="s">
-        <v>52</v>
-      </c>
       <c r="F5" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="G5" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I5" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1986,25 +1986,25 @@
         <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="G6" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I6" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -2015,25 +2015,25 @@
         <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F7" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="G7" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I7" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -2044,25 +2044,25 @@
         <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="G8" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I8" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -2073,25 +2073,25 @@
         <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F9" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="G9" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I9" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -2102,25 +2102,25 @@
         <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E10" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="G10" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I10" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -2131,25 +2131,25 @@
         <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E11" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="G11" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I11" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -2160,25 +2160,25 @@
         <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="G12" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I12" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -2186,28 +2186,28 @@
         <v>18</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>38</v>
+        <v>132</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>129</v>
       </c>
       <c r="F13" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="G13" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I13" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -2215,28 +2215,28 @@
         <v>19</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>39</v>
+        <v>133</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>130</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>131</v>
       </c>
       <c r="G14" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I14" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -2244,28 +2244,28 @@
         <v>20</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>40</v>
+        <v>134</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="G15" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I15" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -2273,28 +2273,28 @@
         <v>21</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E16" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="F16" t="s">
+        <v>76</v>
+      </c>
+      <c r="G16" t="s">
         <v>83</v>
       </c>
-      <c r="G16" t="s">
-        <v>90</v>
-      </c>
       <c r="H16" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I16" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -2302,28 +2302,28 @@
         <v>22</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C17" t="s">
         <v>2</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F17" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G17" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I17" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -2331,28 +2331,28 @@
         <v>23</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F18" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="G18" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I18" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
@@ -2360,28 +2360,28 @@
         <v>24</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C19" t="s">
-        <v>100</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="E19" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="F19" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="G19" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I19" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -2389,28 +2389,28 @@
         <v>25</v>
       </c>
       <c r="B20" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C20" t="s">
+        <v>93</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" t="s">
+        <v>61</v>
+      </c>
+      <c r="F20" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20" t="s">
+        <v>83</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C20" t="s">
-        <v>100</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E20" t="s">
-        <v>67</v>
-      </c>
-      <c r="F20" t="s">
-        <v>87</v>
-      </c>
-      <c r="G20" t="s">
-        <v>90</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>49</v>
-      </c>
       <c r="I20" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -2418,28 +2418,28 @@
         <v>26</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C21" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E21" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F21" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="G21" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I21" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -2447,120 +2447,120 @@
         <v>27</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C22" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E22" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F22" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="G22" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I22" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" t="s">
+        <v>102</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" t="s">
+        <v>103</v>
+      </c>
+      <c r="F23" t="s">
         <v>105</v>
       </c>
-      <c r="B23" t="s">
-        <v>108</v>
-      </c>
-      <c r="C23" t="s">
-        <v>110</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E23" t="s">
-        <v>111</v>
-      </c>
-      <c r="F23" t="s">
-        <v>113</v>
-      </c>
       <c r="G23" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I23" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B24" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" t="s">
+        <v>104</v>
+      </c>
+      <c r="F24" t="s">
         <v>106</v>
       </c>
-      <c r="B24" t="s">
-        <v>109</v>
-      </c>
-      <c r="C24" t="s">
-        <v>110</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E24" t="s">
-        <v>112</v>
-      </c>
-      <c r="F24" t="s">
-        <v>114</v>
-      </c>
       <c r="G24" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I24" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="B25" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C25" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E25" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="F25" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="G25" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix config.yml path resolution and update screener
</commit_message>
<xml_diff>
--- a/tests/Testing.xlsx
+++ b/tests/Testing.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c7d7d98c037d19b/Level 6/Cloud/ACDT CW2 Updated/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="112" documentId="8_{AB4D71AA-F82A-4017-8E7A-B8E1FF7AC13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB2213FE-3847-47D3-9F2D-26636208F9B4}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="8_{AB4D71AA-F82A-4017-8E7A-B8E1FF7AC13D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2475500D-28A0-4231-A0AC-6E663E320073}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0FD93C22-EA38-4C55-8FBA-9A662F17215C}"/>
   </bookViews>
@@ -1496,10 +1496,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58C4BEC0-A8AD-8244-2FDB-36038662FAB9}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E5691BB-5CEC-769B-76F6-2ED2ADBE094E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1526,6 +1526,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>